<commit_message>
convE missing result added
</commit_message>
<xml_diff>
--- a/benchmarking/search_for_best_combination/results.xlsx
+++ b/benchmarking/search_for_best_combination/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/deborahdore/Documents/political-debates-graph-analysis/benchmarking/search_for_best_combination/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{831181EC-42E3-4F42-BF23-48905B3246AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DC9D729-B24F-4941-9178-7771B34C1324}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="26600" xr2:uid="{0963C398-0EAF-144E-8F53-902D2895FD9C}"/>
+    <workbookView xWindow="4280" yWindow="500" windowWidth="46920" windowHeight="26600" xr2:uid="{0963C398-0EAF-144E-8F53-902D2895FD9C}"/>
   </bookViews>
   <sheets>
     <sheet name="Trial 1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="170">
   <si>
     <t>LP HITS@10</t>
   </si>
@@ -538,6 +538,15 @@
   </si>
   <si>
     <t>NOT MORE THAN 0.20 DIFFERENCE BETWEEN LD AND LD</t>
+  </si>
+  <si>
+    <t>0.098853983</t>
+  </si>
+  <si>
+    <t>0.1402067639</t>
+  </si>
+  <si>
+    <t>0.6756550923</t>
   </si>
 </sst>
 </file>
@@ -638,7 +647,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -703,15 +712,6 @@
     <xf numFmtId="2" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -720,6 +720,9 @@
     </xf>
     <xf numFmtId="2" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1109,7 +1112,7 @@
       <c r="H2" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="25" t="s">
         <v>101</v>
       </c>
     </row>
@@ -1138,7 +1141,7 @@
       <c r="H3" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I3" s="22"/>
+      <c r="I3" s="25"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
@@ -1165,7 +1168,7 @@
       <c r="H4" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I4" s="22"/>
+      <c r="I4" s="25"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
@@ -1192,7 +1195,7 @@
       <c r="H7" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I7" s="22" t="s">
+      <c r="I7" s="25" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1221,7 +1224,7 @@
       <c r="H8" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I8" s="22"/>
+      <c r="I8" s="25"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
@@ -1248,7 +1251,7 @@
       <c r="H9" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I9" s="22"/>
+      <c r="I9" s="25"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="F10" s="11"/>
@@ -1269,7 +1272,7 @@
       <c r="H12" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I12" s="22" t="s">
+      <c r="I12" s="25" t="s">
         <v>99</v>
       </c>
     </row>
@@ -1289,7 +1292,7 @@
       <c r="H13" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I13" s="22"/>
+      <c r="I13" s="25"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
@@ -1307,7 +1310,7 @@
       <c r="H14" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="I14" s="22"/>
+      <c r="I14" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
@@ -1325,7 +1328,7 @@
       <c r="H17" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="I17" s="22" t="s">
+      <c r="I17" s="25" t="s">
         <v>100</v>
       </c>
     </row>
@@ -1345,7 +1348,7 @@
       <c r="H18" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="I18" s="22"/>
+      <c r="I18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
@@ -1363,7 +1366,7 @@
       <c r="H19" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="I19" s="22"/>
+      <c r="I19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="G20" s="8"/>
@@ -1402,7 +1405,7 @@
       <c r="H23" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="I23" s="22" t="s">
+      <c r="I23" s="25" t="s">
         <v>106</v>
       </c>
     </row>
@@ -1431,7 +1434,7 @@
       <c r="H24" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="I24" s="22"/>
+      <c r="I24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
@@ -1458,7 +1461,7 @@
       <c r="H25" s="8" t="s">
         <v>105</v>
       </c>
-      <c r="I25" s="22"/>
+      <c r="I25" s="25"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="E26" s="11"/>
@@ -1490,10 +1493,10 @@
       <c r="H28" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="I28" s="22" t="s">
+      <c r="I28" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="J28" s="22"/>
+      <c r="J28" s="25"/>
       <c r="K28" s="9"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
@@ -1521,8 +1524,8 @@
       <c r="H29" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
+      <c r="I29" s="25"/>
+      <c r="J29" s="25"/>
       <c r="K29" s="9"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
@@ -1550,8 +1553,8 @@
       <c r="H30" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
       <c r="K30" s="9"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -1582,7 +1585,7 @@
       <c r="H33" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="I33" s="22" t="s">
+      <c r="I33" s="25" t="s">
         <v>111</v>
       </c>
     </row>
@@ -1611,7 +1614,7 @@
       <c r="H34" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="I34" s="22"/>
+      <c r="I34" s="25"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
@@ -1638,7 +1641,7 @@
       <c r="H35" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="I35" s="22"/>
+      <c r="I35" s="25"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E36" s="11"/>
@@ -1941,6 +1944,15 @@
       </c>
       <c r="C55" s="4" t="s">
         <v>121</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="F55" s="12" t="s">
+        <v>169</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>125</v>
@@ -2279,7 +2291,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D6B6AD7-F64C-7247-AEDD-F4FE3CAA8CE9}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="21.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" style="4" customWidth="1"/>
@@ -2345,12 +2357,12 @@
       <c r="H2" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="I2" s="22" t="s">
+      <c r="I2" s="25" t="s">
         <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="I3" s="22"/>
+      <c r="I3" s="25"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
@@ -2383,19 +2395,19 @@
       <c r="I5" s="7"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="D6" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="E6" s="24" t="s">
+      <c r="E6" s="11" t="s">
         <v>81</v>
       </c>
       <c r="F6" s="6" t="s">
@@ -2412,19 +2424,19 @@
       <c r="H7" s="7"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="D8" s="26" t="s">
+      <c r="D8" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="24" t="s">
         <v>87</v>
       </c>
       <c r="F8" s="6" t="s">
@@ -2442,38 +2454,24 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>132</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="G12" s="6" t="s">
         <v>123</v>
       </c>
     </row>

</xml_diff>